<commit_message>
docs: fold 292 into BUG-004 publish unlock
</commit_message>
<xml_diff>
--- a/docs/ops/チケット棚卸し案_2026-05-02.xlsx
+++ b/docs/ops/チケット棚卸し案_2026-05-02.xlsx
@@ -26,14 +26,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Hearing_Round6_Final" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Cost_Principle" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Publish0_NarrowUnlock" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_2026_05_03_PMO" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_Final_JP'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_ACTIVE_Detail'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_ACTIVE_Detail'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_KEEP_Detail'!$A$1:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_HOLD_OBSOLETE'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_Rules_Detail'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Claude_Prompt'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Claude_Prompt'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_NewCandidate_GCP_Codex'!$A$1:$B$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'00_UserReview'!$A$1:$C$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'01_AllTickets'!$A$1:$K$56</definedName>
@@ -47,6 +48,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'09_Hearing_Round6_Final'!$A$1:$C$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'10_Cost_Principle'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'07_Publish0_NarrowUnlock'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'08_2026_05_03_PMO'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -542,7 +544,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1751,7 +1753,7 @@
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="47" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2008,8 +2010,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2130,7 +2132,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2233,7 +2235,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2332,17 +2334,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2353,168 +2355,337 @@
       </c>
       <c r="B1" s="9" t="inlineStr">
         <is>
-          <t>チケット名</t>
+          <t>?????</t>
         </is>
       </c>
       <c r="C1" s="9" t="inlineStr">
         <is>
-          <t>優先度</t>
+          <t>???</t>
         </is>
       </c>
       <c r="D1" s="9" t="inlineStr">
         <is>
-          <t>扱い</t>
+          <t>??</t>
         </is>
       </c>
       <c r="E1" s="9" t="inlineStr">
         <is>
-          <t>なぜ重要か</t>
+          <t>?????</t>
         </is>
       </c>
       <c r="F1" s="9" t="inlineStr">
         <is>
-          <t>次にやること</t>
+          <t>??????</t>
         </is>
       </c>
       <c r="G1" s="9" t="inlineStr">
         <is>
-          <t>close条件</t>
+          <t>close??</t>
         </is>
       </c>
       <c r="H1" s="9" t="inlineStr">
         <is>
-          <t>禁止/注意</t>
+          <t>??/??</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>BUG-003</t>
+          <t>BUG-004+291</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>WP status mutation audit</t>
+          <t>publish=0???? + narrow publish-path unlock</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>P1候補</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>ACTIVE候補 1</t>
+          <t>ACTIVE 1???</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>公開状態が勝手に変わった疑い。publish済み記事がdraft/private/pending等に戻る事故があると、サイトの公開復旧・信頼性に直結する。</t>
+          <t>???????????user??????????????????????????????????publish path?????????</t>
         </is>
       </c>
       <c r="F2" s="10" t="inlineStr">
         <is>
-          <t>直近24〜72hのWP status変化、WP REST更新ログ、guarded-publish/publish-notice周辺のstatus更新pathをread-onlyで確認する。既存publishをdraft/privateへ戻す処理が存在しない、または十分guardされていることを確認する。</t>
+          <t>read-only?publish=0??????277/289/290/4-tier/duplicate/backlog/freshness/body_contract/subtype/numeric/placeholder/source facts?????????unlock??????????????292 body_contract_fail durable ledger?????????</t>
         </is>
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>問題なしを証拠付きで確認できた、または原因を特定して修正・verifyできた場合のみDONE。証拠なしはDONE禁止でP1_REVIEWまたはOBSERVE継続。</t>
+          <t>?????(YOSHILOVER???source_url?subtype/template_key high confidence?numeric/body pass?placeholder???silent skip???title???review/hold????)????????publish????????????body_contract_fail???????????ledger/log?????</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>本番変更なし。deploy/env/flag/Scheduler/SEO/source/Gemini/mail変更禁止。</t>
+          <t>publish gate?????postgame strict/stale/duplicate??????noindex???review threshold?????mail?????ticket???292??ACTIVE?????</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>BUG-004 + 291</t>
+          <t>282-COST</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>silent skip / ???? / YOSHILOVER?????? / ???????? / publish=0????</t>
+          <t>flag ON? preflight active rejection??</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>P1候補</t>
+          <t>OBSERVE</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>ACTIVE候補 2</t>
+          <t>OBSERVE</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>??????????publish/review/hold/skip/error??????????????YOSHILOVER???source??????????publish=0??????user?????????????????????????</t>
+          <t>282?flag ON???????????????????????????</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>????????read-only??????publish=0???277 title quality?289 post_gen_validate?290 weak title rescue???4-tier strict?duplicate/backlog/freshness?body_contract?subtype????numeric guard?placeholder?source facts??????????????????????????????publish path???narrow unlock??????</t>
+          <t>preflight active rejection?????silent skip?Gemini??mail storm?????</t>
         </is>
       </c>
       <c r="G3" s="10" t="inlineStr">
         <is>
-          <t>??run?unaccounted candidate?0?skip/hold/review???log/ledger/state row????YOSHILOVER????????????????(YOSHILOVER???source_url?subtype/template_key high confidence?numeric/body pass?placeholder???title???review/hold????)????????publish???????????DONE???</t>
+          <t>?????????????????????????</t>
         </is>
       </c>
       <c r="H3" s="10" t="inlineStr">
         <is>
-          <t>publish gate??????????noindex???review threshold???????mail??????292 body_contract fail?????????ledger/log????????????</t>
+          <t>?????env remove?user?????????</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>NEW_CANDIDATE</t>
+          <t>298-Phase3</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>GCP Codex WP本文修正プレビュー v0</t>
+          <t>5/3 19:35 JST 24h gate??</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>P1候補/次ACTIVE候補</t>
+          <t>OBSERVE</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>まだACTIVEではないが早めにやりたい</t>
+          <t>OBSERVE</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>本文品質を早く見たい。preview-onlyならデグレリスクを抑えてGCP Codexの実力を確認できる。</t>
+          <t>24h gate?PASS/FAIL??????</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>postgameまたはfarm_result少数で、元本文と修正文候補を比較できるartifactを出す。</t>
+          <t>5/3 19:35 JST????</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>WP本文変更なし、publish変更なし、Gemini原則0で品質確認できる。</t>
+          <t>PASS/FAIL/rollback???????</t>
         </is>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t>本番本文を書き換えない。自由作文させない。</t>
+          <t>????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>WP plugin upload</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>USER_DECISION_REQUIRED</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>user????</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>WP admin upload?????????????user???</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>upload????OK/HOLD/REJECT????</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>user?OK?????????</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>publish=0?????????</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:H5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>BUG-004+291 publish=0???? + narrow publish-path unlock ?1??292 body_contract_fail durable ledger????????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>OBSERVE</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>282-COST flag ON??preflight active rejection?? / 298 5/3 19:35 JST 24h gate??????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>USER_DECISION_REQUIRED</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>245 WP plugin upload???</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>???</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>277/279/278/280 title/mail/summary??234/247/250/256/254/295 ???????subtype??246-MKT/195/197/281 ????????????230/288/251/252/274/296/238 HOLD/OBSOLETE???</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>??????????????????292??ACTIVE??publish gate?????postgame strict/stale/duplicate??????noindex???review threshold?????mail???body_contract_fail??????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>????????????????publish path????</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>publish????</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>YOSHILOVER???source_url???subtype/template_key high confidence?numeric guard pass?body_contract pass?placeholder???silent skip???title???????????????review/hold?????</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>??Claude????</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>??Claude?BUG-004+291????????????publish=0????+narrow publish-path unlock?BUG-004+291???????????????????292 body_contract_fail durable ledger?????ACTIVE?????????????????????????????????read-only?publish=0??????????unlock???????????????????</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2531,8 +2702,8 @@
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2985,7 +3156,7 @@
     <col width="27" customWidth="1" min="1" max="1"/>
     <col width="54" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3202,7 +3373,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3349,11 +3520,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3428,8 +3599,20 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-03 ??Claude??????</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>?????????Claude?BUG-004+291???????????????publish=0???? + narrow publish-path unlock??BUG-004+291??????????????????????292 body_contract_fail durable ledger?????ACTIVE?????BUG-004+291????????????????????????ACTIVE?BUG-004+291???OBSERVE?282-COST?298-Phase3?USER_DECISION_REQUIRED?245 WP plugin upload???publish gate?????postgame strict/stale/duplicate??????noindex???review threshold???????mail????????????body_contract_fail???????????????read-only?publish=0??????????unlock???????????????????</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3444,7 +3627,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3656,7 +3839,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3879,16 +4062,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
     <col width="31" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>